<commit_message>
Add new Update Cart Test
</commit_message>
<xml_diff>
--- a/src/test/resources/search.xlsx
+++ b/src/test/resources/search.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coder\Selenium\Totoday\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29EBD44E-B164-4C5B-A07D-C60DE8E92E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA8954B-9C06-44A1-AB80-EACD8DE178AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{3DE178C0-15D6-4806-B357-75CE9BEFD093}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{3DE178C0-15D6-4806-B357-75CE9BEFD093}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="SearchData" sheetId="1" r:id="rId1"/>
+    <sheet name="CategoryData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -112,7 +112,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,18 +137,6 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF808080"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF61AFE1"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -170,18 +158,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -518,12 +507,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{761588E0-63B1-4C2B-8FB5-42753A584D18}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="59.453125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" ht="28" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -531,59 +522,59 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -595,53 +586,57 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C231D0FA-AE64-4CA1-8CFB-BA67BBEC42DA}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.81640625" customWidth="1"/>
+    <col min="2" max="2" width="47.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>